<commit_message>
feat: improve export capture and workbook data
</commit_message>
<xml_diff>
--- a/work/处理表格.xlsx
+++ b/work/处理表格.xlsx
@@ -101,12 +101,24 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="21">
   <si>
     <t>交易单号</t>
   </si>
   <si>
     <t>商户单号</t>
+  </si>
+  <si>
+    <t>交易金额</t>
+  </si>
+  <si>
+    <t>交易时间</t>
+  </si>
+  <si>
+    <t>咨询时间</t>
+  </si>
+  <si>
+    <t>问题描述</t>
   </si>
   <si>
     <t>退款情况</t>
@@ -1319,22 +1331,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:Q4"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="3"/>
   <cols>
     <col min="1" max="1" width="32.1111111111111" customWidth="1"/>
     <col min="2" max="2" width="18.6666666666667" customWidth="1"/>
-    <col min="3" max="3" width="8.33333333333333" customWidth="1"/>
-    <col min="4" max="4" width="20.8888888888889" customWidth="1"/>
-    <col min="5" max="5" width="19.7777777777778" customWidth="1"/>
-    <col min="6" max="6" width="20.3333333333333" customWidth="1"/>
-    <col min="7" max="7" width="24.1111111111111" customWidth="1"/>
-    <col min="8" max="8" width="18.3333333333333" customWidth="1"/>
-    <col min="9" max="10" width="9.22222222222222" customWidth="1"/>
-    <col min="11" max="11" width="8.33333333333333" customWidth="1"/>
+    <col min="3" max="7" width="8.33333333333333" customWidth="1"/>
+    <col min="8" max="8" width="20.8888888888889" customWidth="1"/>
+    <col min="9" max="9" width="19.7777777777778" customWidth="1"/>
+    <col min="10" max="10" width="20.3333333333333" customWidth="1"/>
+    <col min="11" max="11" width="24.1111111111111" customWidth="1"/>
+    <col min="12" max="12" width="18.3333333333333" customWidth="1"/>
+    <col min="13" max="14" width="9.22222222222222" customWidth="1"/>
+    <col min="15" max="15" width="8.33333333333333" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:17">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1359,92 +1371,116 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
-        <v>8</v>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>8</v>
+        <v>11</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
-    <row r="2" ht="73.05" spans="1:13">
+    <row r="2" ht="73.05" spans="1:17">
       <c r="A2" s="3" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="4">
+        <v>14</v>
+      </c>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="4">
         <v>46165.8291666667</v>
       </c>
-      <c r="E2" s="4">
+      <c r="I2" s="4">
         <v>46165.8388888889</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" t="str">
+      <c r="J2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" t="str">
         <f>_xlfn.DISPIMG("ID_8E3C3DAA516B482F91FC37E1C56D9C9B",1)</f>
         <v>=DISPIMG("ID_8E3C3DAA516B482F91FC37E1C56D9C9B",1)</v>
       </c>
     </row>
-    <row r="3" ht="73.05" spans="1:13">
+    <row r="3" ht="73.05" spans="1:17">
       <c r="A3" s="5" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="4">
+        <v>18</v>
+      </c>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="4">
         <v>46163.5125</v>
       </c>
-      <c r="E3" s="4">
+      <c r="I3" s="4">
         <v>46163.5215277778</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="I3" t="str">
+      <c r="J3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="M3" t="str">
         <f>_xlfn.DISPIMG("ID_5F383231F134484DBF500EE09062F477",1)</f>
         <v>=DISPIMG("ID_5F383231F134484DBF500EE09062F477",1)</v>
       </c>
     </row>
-    <row r="4" ht="73.05" spans="1:13">
+    <row r="4" ht="73.05" spans="1:17">
       <c r="A4" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="H4" s="4">
+        <v>46162.7680555556</v>
+      </c>
+      <c r="I4" s="4">
+        <v>46162.84375</v>
+      </c>
+      <c r="J4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="4">
-        <v>46162.7680555556</v>
-      </c>
-      <c r="E4" s="4">
-        <v>46162.84375</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="I4" t="str">
+      <c r="M4" t="str">
         <f>_xlfn.DISPIMG("ID_2AD7661407C74EF688435F5AC8652145",1)</f>
         <v>=DISPIMG("ID_2AD7661407C74EF688435F5AC8652145",1)</v>
       </c>

</xml_diff>

<commit_message>
feat: add configurable excel field extraction
</commit_message>
<xml_diff>
--- a/work/处理表格.xlsx
+++ b/work/处理表格.xlsx
@@ -101,7 +101,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="22">
   <si>
     <t>交易单号</t>
   </si>
@@ -113,6 +113,9 @@
   </si>
   <si>
     <t>交易时间</t>
+  </si>
+  <si>
+    <t>咨询原因</t>
   </si>
   <si>
     <t>咨询时间</t>
@@ -1331,22 +1334,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:Q4"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="3"/>
   <cols>
     <col min="1" max="1" width="32.1111111111111" customWidth="1"/>
     <col min="2" max="2" width="18.6666666666667" customWidth="1"/>
-    <col min="3" max="7" width="8.33333333333333" customWidth="1"/>
-    <col min="8" max="8" width="20.8888888888889" customWidth="1"/>
-    <col min="9" max="9" width="19.7777777777778" customWidth="1"/>
-    <col min="10" max="10" width="20.3333333333333" customWidth="1"/>
-    <col min="11" max="11" width="24.1111111111111" customWidth="1"/>
-    <col min="12" max="12" width="18.3333333333333" customWidth="1"/>
-    <col min="13" max="14" width="9.22222222222222" customWidth="1"/>
-    <col min="15" max="15" width="8.33333333333333" customWidth="1"/>
+    <col min="3" max="8" width="8.33333333333333" customWidth="1"/>
+    <col min="9" max="9" width="20.8888888888889" customWidth="1"/>
+    <col min="10" max="10" width="19.7777777777778" customWidth="1"/>
+    <col min="11" max="11" width="20.3333333333333" customWidth="1"/>
+    <col min="12" max="12" width="24.1111111111111" customWidth="1"/>
+    <col min="13" max="13" width="18.3333333333333" customWidth="1"/>
+    <col min="14" max="15" width="9.22222222222222" customWidth="1"/>
+    <col min="16" max="16" width="8.33333333333333" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:18">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1383,104 +1386,110 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="2" ht="73.05" spans="1:17">
+    <row r="2" ht="73.05" spans="1:18">
       <c r="A2" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
-      <c r="G2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H2" s="4">
+      <c r="G2" s="1"/>
+      <c r="H2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="4">
         <v>46165.8291666667</v>
       </c>
-      <c r="I2" s="4">
+      <c r="J2" s="4">
         <v>46165.8388888889</v>
       </c>
-      <c r="J2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="K2" s="1"/>
+      <c r="K2" s="1" t="s">
+        <v>17</v>
+      </c>
       <c r="L2" s="1"/>
-      <c r="M2" t="str">
+      <c r="M2" s="1"/>
+      <c r="N2" t="str">
         <f>_xlfn.DISPIMG("ID_8E3C3DAA516B482F91FC37E1C56D9C9B",1)</f>
         <v>=DISPIMG("ID_8E3C3DAA516B482F91FC37E1C56D9C9B",1)</v>
       </c>
     </row>
-    <row r="3" ht="73.05" spans="1:17">
+    <row r="3" ht="73.05" spans="1:18">
       <c r="A3" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
-      <c r="G3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" s="4">
+      <c r="G3" s="1"/>
+      <c r="H3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="4">
         <v>46163.5125</v>
       </c>
-      <c r="I3" s="4">
+      <c r="J3" s="4">
         <v>46163.5215277778</v>
       </c>
-      <c r="J3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="M3" t="str">
+      <c r="K3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="N3" t="str">
         <f>_xlfn.DISPIMG("ID_5F383231F134484DBF500EE09062F477",1)</f>
         <v>=DISPIMG("ID_5F383231F134484DBF500EE09062F477",1)</v>
       </c>
     </row>
-    <row r="4" ht="73.05" spans="1:17">
+    <row r="4" ht="73.05" spans="1:18">
       <c r="A4" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
-      <c r="G4" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H4" s="4">
+      <c r="G4" s="1"/>
+      <c r="H4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" s="4">
         <v>46162.7680555556</v>
       </c>
-      <c r="I4" s="4">
+      <c r="J4" s="4">
         <v>46162.84375</v>
       </c>
-      <c r="J4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="M4" t="str">
+      <c r="K4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="N4" t="str">
         <f>_xlfn.DISPIMG("ID_2AD7661407C74EF688435F5AC8652145",1)</f>
         <v>=DISPIMG("ID_2AD7661407C74EF688435F5AC8652145",1)</v>
       </c>

</xml_diff>